<commit_message>
Add a Notes sheet to the two workbooks that had none
The commute survey and the sales explorer were the only workbooks without one. Each Notes sheet
now says the data was written for the book and gives the scenario, the question and what is raw
about the file, as the others do. The sheets were added to the workbook packages directly, so every
other part, including the sales explorer's six charts, is byte for byte as before. data/README.md
no longer lists the two as exceptions.
</commit_message>
<xml_diff>
--- a/data/capstone-commute-mode-by-region.xlsx
+++ b/data/capstone-commute-mode-by-region.xlsx
@@ -11,6 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Questionnaire" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sampling" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Codebook" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes" sheetId="5" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -19210,4 +19211,70 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="70" customWidth="1" min="1" max="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>A teaching dataset written for the book. It holds a stratified survey of residents about how they get to work or study, and the residents and their answers are made up.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Question: is commute mode related to the kind of area a resident lives in (Urban Core, Inner Suburb, Outer Suburb or Rural)?</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Design: 200 residents were drawn at random from each area type, so the area totals do not reflect population shares. The Sampling sheet has the details.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>This export is deliberately raw. The area labels arrive in mixed case, two rows are duplicated, and five responses are missing the area or the commute mode.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Cleaning guide: standardize the area label, drop duplicate rows, then drop responses missing either of the two variables under test.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Age and the 1-to-7 commute satisfaction rating are carried for a check near the end of the notebook.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>